<commit_message>
Changes on regression testing. Adding data-testid on UI elements.
</commit_message>
<xml_diff>
--- a/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
+++ b/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\testing\PIMS.Tests.Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A607B79-8FC2-4359-ACDD-70FFC6886FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D48D8B60-00C0-438B-9F65-2B3B68325284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="19" activeTab="32" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="3" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4227" uniqueCount="2406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4266" uniqueCount="2413">
   <si>
     <t>FirstName</t>
   </si>
@@ -7300,6 +7300,27 @@
   </si>
   <si>
     <t>Fee Simple - MoTT;Closed Road</t>
+  </si>
+  <si>
+    <t>Compensation to test lease errors</t>
+  </si>
+  <si>
+    <t>Testing lease- compensation errors</t>
+  </si>
+  <si>
+    <t>Automation Functional Testing - Note Test Property 1;Automation Functional Testing - Note Test Property 2;Automation Functional Testing - Note Test Property 3</t>
+  </si>
+  <si>
+    <t>Property - Edit note</t>
+  </si>
+  <si>
+    <t>Property - Create new notes</t>
+  </si>
+  <si>
+    <t>Lease compensation errors</t>
+  </si>
+  <si>
+    <t>Lease minimum for Notes</t>
   </si>
 </sst>
 </file>
@@ -7396,7 +7417,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -7482,6 +7503,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -10649,7 +10671,7 @@
       </c>
       <c r="N3" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="O3" s="4">
         <v>45318</v>
@@ -10887,7 +10909,7 @@
       </c>
       <c r="N5" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="O5" s="4">
         <v>45318</v>
@@ -11112,7 +11134,7 @@
       </c>
       <c r="N7" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="O7" s="4">
         <v>45318</v>
@@ -11685,7 +11707,7 @@
       </c>
       <c r="N12" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="O12" s="4">
         <v>45318</v>
@@ -12028,7 +12050,7 @@
       </c>
       <c r="N15" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="O15" s="4">
         <v>45318</v>
@@ -15098,7 +15120,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01CC3795-F36B-4D0F-8244-A4F4C3935686}">
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="50.44140625" bestFit="1" customWidth="1"/>
@@ -15635,6 +15657,57 @@
       </c>
       <c r="V9">
         <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>2406</v>
+      </c>
+      <c r="B10" s="37"/>
+      <c r="E10" t="s">
+        <v>490</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1821</v>
+      </c>
+      <c r="G10" s="4">
+        <v>45569</v>
+      </c>
+      <c r="K10" t="s">
+        <v>2407</v>
+      </c>
+      <c r="L10" t="s">
+        <v>1576</v>
+      </c>
+      <c r="M10" s="53" t="s">
+        <v>1872</v>
+      </c>
+      <c r="N10" s="53" t="s">
+        <v>895</v>
+      </c>
+      <c r="O10" s="53" t="s">
+        <v>1813</v>
+      </c>
+      <c r="P10" s="53" t="s">
+        <v>1814</v>
+      </c>
+      <c r="Q10" s="53" t="s">
+        <v>796</v>
+      </c>
+      <c r="R10" s="53" t="b">
+        <v>0</v>
+      </c>
+      <c r="S10" s="53" t="s">
+        <v>1395</v>
+      </c>
+      <c r="T10" s="53" t="s">
+        <v>1815</v>
+      </c>
+      <c r="U10">
+        <v>0</v>
+      </c>
+      <c r="V10">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -16762,7 +16835,7 @@
       </c>
       <c r="F4" s="4">
         <f ca="1">TODAY()</f>
-        <v>45926</v>
+        <v>45951</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
@@ -25968,7 +26041,7 @@
 
 <file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68E0191B-A695-44B6-B8DB-539DF91B46C4}">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32.77734375" bestFit="1" customWidth="1"/>
@@ -26076,6 +26149,22 @@
         <v>2276</v>
       </c>
       <c r="B13" t="s">
+        <v>2277</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>2410</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2408</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>2409</v>
+      </c>
+      <c r="B15" t="s">
         <v>2277</v>
       </c>
     </row>
@@ -28081,7 +28170,7 @@
         <v>1</v>
       </c>
       <c r="AW8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX8">
         <v>1</v>
@@ -29133,7 +29222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:104" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>2194</v>
       </c>
@@ -29258,7 +29347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:104" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:105" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>2194</v>
       </c>
@@ -29383,15 +29472,260 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:104" x14ac:dyDescent="0.3">
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
-    </row>
-    <row r="20" spans="1:104" x14ac:dyDescent="0.3">
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
-    </row>
-    <row r="21" spans="1:104" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:105" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>2411</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1018</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1017</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1985</v>
+      </c>
+      <c r="E19" t="s">
+        <v>490</v>
+      </c>
+      <c r="I19" t="s">
+        <v>2379</v>
+      </c>
+      <c r="J19" s="4">
+        <v>45209</v>
+      </c>
+      <c r="L19" s="8">
+        <v>0</v>
+      </c>
+      <c r="M19" s="8">
+        <v>0</v>
+      </c>
+      <c r="O19" t="s">
+        <v>191</v>
+      </c>
+      <c r="P19" t="s">
+        <v>1803</v>
+      </c>
+      <c r="R19" t="s">
+        <v>1804</v>
+      </c>
+      <c r="T19" t="s">
+        <v>1805</v>
+      </c>
+      <c r="AI19" t="s">
+        <v>297</v>
+      </c>
+      <c r="AJ19" t="s">
+        <v>297</v>
+      </c>
+      <c r="AK19" t="s">
+        <v>297</v>
+      </c>
+      <c r="AM19">
+        <v>0</v>
+      </c>
+      <c r="AN19">
+        <v>0</v>
+      </c>
+      <c r="AO19" s="2">
+        <v>21</v>
+      </c>
+      <c r="AP19">
+        <v>0</v>
+      </c>
+      <c r="AQ19">
+        <v>0</v>
+      </c>
+      <c r="AR19">
+        <v>0</v>
+      </c>
+      <c r="AS19">
+        <v>0</v>
+      </c>
+      <c r="AT19">
+        <v>0</v>
+      </c>
+      <c r="AU19">
+        <v>1</v>
+      </c>
+      <c r="AV19">
+        <v>4</v>
+      </c>
+      <c r="AW19">
+        <v>0</v>
+      </c>
+      <c r="AX19">
+        <v>0</v>
+      </c>
+      <c r="AY19">
+        <v>0</v>
+      </c>
+      <c r="AZ19">
+        <v>0</v>
+      </c>
+      <c r="BA19">
+        <v>0</v>
+      </c>
+      <c r="BB19">
+        <v>2</v>
+      </c>
+      <c r="BC19">
+        <v>2</v>
+      </c>
+      <c r="BM19">
+        <v>0</v>
+      </c>
+      <c r="CQ19">
+        <v>0</v>
+      </c>
+      <c r="CS19">
+        <v>0</v>
+      </c>
+      <c r="CT19">
+        <v>0</v>
+      </c>
+      <c r="CU19">
+        <v>0</v>
+      </c>
+      <c r="CV19">
+        <v>0</v>
+      </c>
+      <c r="CW19">
+        <v>0</v>
+      </c>
+      <c r="CX19">
+        <v>0</v>
+      </c>
+      <c r="CY19">
+        <v>9</v>
+      </c>
+      <c r="CZ19">
+        <v>1</v>
+      </c>
+      <c r="DA19">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:105" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>2412</v>
+      </c>
+      <c r="E20" t="s">
+        <v>490</v>
+      </c>
+      <c r="I20" t="s">
+        <v>2379</v>
+      </c>
+      <c r="L20" s="8">
+        <v>0</v>
+      </c>
+      <c r="M20" s="8">
+        <v>0</v>
+      </c>
+      <c r="O20" t="s">
+        <v>191</v>
+      </c>
+      <c r="P20" t="s">
+        <v>1803</v>
+      </c>
+      <c r="R20" t="s">
+        <v>1804</v>
+      </c>
+      <c r="T20" t="s">
+        <v>1805</v>
+      </c>
+      <c r="AI20" t="s">
+        <v>297</v>
+      </c>
+      <c r="AJ20" t="s">
+        <v>297</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>297</v>
+      </c>
+      <c r="AM20">
+        <v>0</v>
+      </c>
+      <c r="AN20">
+        <v>0</v>
+      </c>
+      <c r="AO20" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP20">
+        <v>0</v>
+      </c>
+      <c r="AQ20">
+        <v>0</v>
+      </c>
+      <c r="AR20">
+        <v>0</v>
+      </c>
+      <c r="AS20">
+        <v>0</v>
+      </c>
+      <c r="AT20">
+        <v>0</v>
+      </c>
+      <c r="AU20">
+        <v>0</v>
+      </c>
+      <c r="AV20">
+        <v>0</v>
+      </c>
+      <c r="AW20">
+        <v>0</v>
+      </c>
+      <c r="AX20">
+        <v>0</v>
+      </c>
+      <c r="AY20">
+        <v>0</v>
+      </c>
+      <c r="AZ20">
+        <v>0</v>
+      </c>
+      <c r="BA20">
+        <v>0</v>
+      </c>
+      <c r="BB20">
+        <v>0</v>
+      </c>
+      <c r="BC20">
+        <v>0</v>
+      </c>
+      <c r="BM20">
+        <v>0</v>
+      </c>
+      <c r="CQ20">
+        <v>0</v>
+      </c>
+      <c r="CS20">
+        <v>0</v>
+      </c>
+      <c r="CT20">
+        <v>0</v>
+      </c>
+      <c r="CU20">
+        <v>0</v>
+      </c>
+      <c r="CV20">
+        <v>0</v>
+      </c>
+      <c r="CW20">
+        <v>0</v>
+      </c>
+      <c r="CX20">
+        <v>0</v>
+      </c>
+      <c r="CY20">
+        <v>0</v>
+      </c>
+      <c r="CZ20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:105" x14ac:dyDescent="0.3">
       <c r="L21" s="8"/>
       <c r="M21" s="8"/>
     </row>

</xml_diff>

<commit_message>
PSP-10924 - Changes based on Regression on UAT
</commit_message>
<xml_diff>
--- a/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
+++ b/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\testing\PIMS.Tests.Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{592CDA47-D6A6-4165-BCB0-9D09518CEB75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C91D6A-C260-45BD-A3EE-C6D4F062DF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="31" activeTab="34" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="3" r:id="rId1"/>
@@ -7287,9 +7287,6 @@
     <t>010-764-135;015-069-940;007-095-333</t>
   </si>
   <si>
-    <t>005-565-383;015-069-940;-131.339444, 52.308056</t>
-  </si>
-  <si>
     <t>026-172-674</t>
   </si>
   <si>
@@ -7381,6 +7378,9 @@
   </si>
   <si>
     <t>002-256-525;90172682;002-406-349</t>
+  </si>
+  <si>
+    <t>005-565-383;001-646-435;-131.339444, 52.308056</t>
   </si>
 </sst>
 </file>
@@ -10730,7 +10730,7 @@
       </c>
       <c r="N3" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="O3" s="4">
         <v>45318</v>
@@ -10968,7 +10968,7 @@
       </c>
       <c r="N5" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="O5" s="4">
         <v>45318</v>
@@ -11193,7 +11193,7 @@
       </c>
       <c r="N7" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="O7" s="4">
         <v>45318</v>
@@ -11766,7 +11766,7 @@
       </c>
       <c r="N12" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="O12" s="4">
         <v>45318</v>
@@ -12109,7 +12109,7 @@
       </c>
       <c r="N15" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="O15" s="4">
         <v>45318</v>
@@ -16894,7 +16894,7 @@
       </c>
       <c r="F4" s="4">
         <f ca="1">TODAY()</f>
-        <v>45982</v>
+        <v>45988</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
@@ -19217,7 +19217,7 @@
         <v>2377</v>
       </c>
       <c r="U12" t="s">
-        <v>2403</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
@@ -19371,7 +19371,7 @@
         <v>2373</v>
       </c>
       <c r="U26" t="s">
-        <v>2401</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.3">
@@ -19487,7 +19487,7 @@
         <v>90172682</v>
       </c>
       <c r="D35" t="s">
-        <v>2431</v>
+        <v>2430</v>
       </c>
       <c r="E35" t="s">
         <v>2228</v>
@@ -19517,7 +19517,7 @@
         <v>2294</v>
       </c>
       <c r="U35" t="s">
-        <v>2432</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.3">
@@ -19540,7 +19540,7 @@
         <v>2375</v>
       </c>
       <c r="U37" t="s">
-        <v>2402</v>
+        <v>2401</v>
       </c>
     </row>
     <row r="38" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
@@ -20889,7 +20889,7 @@
         <v>1189</v>
       </c>
       <c r="D2" t="s">
-        <v>2424</v>
+        <v>2423</v>
       </c>
       <c r="E2" t="s">
         <v>1213</v>
@@ -20904,7 +20904,7 @@
         <v>2158</v>
       </c>
       <c r="J2" t="s">
-        <v>2418</v>
+        <v>2417</v>
       </c>
       <c r="K2" t="s">
         <v>1195</v>
@@ -20942,7 +20942,7 @@
         <v>1190</v>
       </c>
       <c r="D3" t="s">
-        <v>2425</v>
+        <v>2424</v>
       </c>
       <c r="E3" t="s">
         <v>1191</v>
@@ -20957,7 +20957,7 @@
         <v>1194</v>
       </c>
       <c r="J3" t="s">
-        <v>2419</v>
+        <v>2418</v>
       </c>
       <c r="K3" t="s">
         <v>2157</v>
@@ -21010,7 +21010,7 @@
         <v>1223</v>
       </c>
       <c r="J4" t="s">
-        <v>2420</v>
+        <v>2419</v>
       </c>
       <c r="K4" t="s">
         <v>1225</v>
@@ -21048,7 +21048,7 @@
         <v>1278</v>
       </c>
       <c r="D5" t="s">
-        <v>2426</v>
+        <v>2425</v>
       </c>
       <c r="E5" t="s">
         <v>1213</v>
@@ -21063,7 +21063,7 @@
         <v>2225</v>
       </c>
       <c r="J5" t="s">
-        <v>2421</v>
+        <v>2420</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -21110,7 +21110,7 @@
         <v>2337</v>
       </c>
       <c r="J6" t="s">
-        <v>2422</v>
+        <v>2421</v>
       </c>
       <c r="K6" t="s">
         <v>2338</v>
@@ -21166,10 +21166,10 @@
         <v>2307</v>
       </c>
       <c r="J7" t="s">
-        <v>2423</v>
+        <v>2422</v>
       </c>
       <c r="K7" t="s">
-        <v>2427</v>
+        <v>2426</v>
       </c>
       <c r="L7" s="14" t="s">
         <v>2315</v>
@@ -21216,13 +21216,13 @@
         <v>2306</v>
       </c>
       <c r="I8" t="s">
+        <v>2427</v>
+      </c>
+      <c r="J8" t="s">
         <v>2428</v>
       </c>
-      <c r="J8" t="s">
+      <c r="K8" t="s">
         <v>2429</v>
-      </c>
-      <c r="K8" t="s">
-        <v>2430</v>
       </c>
       <c r="L8" t="s">
         <v>2316</v>
@@ -27985,7 +27985,7 @@
     </row>
     <row r="6" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>2416</v>
+        <v>2415</v>
       </c>
       <c r="E6" t="s">
         <v>490</v>
@@ -29854,7 +29854,7 @@
     </row>
     <row r="21" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>2404</v>
+        <v>2403</v>
       </c>
       <c r="E21" t="s">
         <v>246</v>
@@ -29987,7 +29987,7 @@
     </row>
     <row r="22" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>2409</v>
+        <v>2408</v>
       </c>
       <c r="E22" t="s">
         <v>246</v>
@@ -30098,7 +30098,7 @@
     </row>
     <row r="23" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>2405</v>
+        <v>2404</v>
       </c>
       <c r="E23" t="s">
         <v>246</v>
@@ -30231,7 +30231,7 @@
     </row>
     <row r="24" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>2406</v>
+        <v>2405</v>
       </c>
       <c r="E24" t="s">
         <v>246</v>
@@ -30391,7 +30391,7 @@
     </row>
     <row r="25" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>2410</v>
+        <v>2409</v>
       </c>
       <c r="E25" t="s">
         <v>246</v>
@@ -30516,7 +30516,7 @@
     </row>
     <row r="26" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>2407</v>
+        <v>2406</v>
       </c>
       <c r="E26" t="s">
         <v>246</v>
@@ -30729,7 +30729,7 @@
     </row>
     <row r="27" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>2411</v>
+        <v>2410</v>
       </c>
       <c r="E27" t="s">
         <v>246</v>
@@ -30853,7 +30853,7 @@
     </row>
     <row r="28" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>2408</v>
+        <v>2407</v>
       </c>
       <c r="E28" t="s">
         <v>246</v>
@@ -30989,7 +30989,7 @@
     </row>
     <row r="29" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>2412</v>
+        <v>2411</v>
       </c>
       <c r="F29" s="4"/>
       <c r="J29" s="4"/>
@@ -31102,7 +31102,7 @@
     </row>
     <row r="30" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>2413</v>
+        <v>2412</v>
       </c>
       <c r="E30" t="s">
         <v>246</v>
@@ -31235,7 +31235,7 @@
     </row>
     <row r="31" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>2414</v>
+        <v>2413</v>
       </c>
       <c r="F31" s="4"/>
       <c r="J31" s="4"/>
@@ -31345,7 +31345,7 @@
     </row>
     <row r="32" spans="1:97" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>2415</v>
+        <v>2414</v>
       </c>
       <c r="L32" s="8">
         <v>0</v>
@@ -31354,7 +31354,7 @@
         <v>0</v>
       </c>
       <c r="P32" t="s">
-        <v>658</v>
+        <v>2378</v>
       </c>
       <c r="AA32" t="s">
         <v>297</v>
@@ -31566,7 +31566,7 @@
     </row>
     <row r="34" spans="1:96" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>2417</v>
+        <v>2416</v>
       </c>
       <c r="E34" t="s">
         <v>490</v>

</xml_diff>

<commit_message>
Automation test set updates
</commit_message>
<xml_diff>
--- a/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
+++ b/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\testing\PIMS.Tests.Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76CFF24A-761C-4CF9-BD8F-7FFB1C75A529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9CE74F-956C-4F87-B318-F1501094476B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="19" activeTab="31" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="3" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4417" uniqueCount="2441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4420" uniqueCount="2441">
   <si>
     <t>FirstName</t>
   </si>
@@ -10754,7 +10754,7 @@
       </c>
       <c r="N3" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="O3" s="4">
         <v>45318</v>
@@ -10992,7 +10992,7 @@
       </c>
       <c r="N5" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="O5" s="4">
         <v>45318</v>
@@ -11217,7 +11217,7 @@
       </c>
       <c r="N7" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="O7" s="4">
         <v>45318</v>
@@ -11790,7 +11790,7 @@
       </c>
       <c r="N12" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="O12" s="4">
         <v>45318</v>
@@ -12133,7 +12133,7 @@
       </c>
       <c r="N15" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="O15" s="4">
         <v>45318</v>
@@ -16918,7 +16918,7 @@
       </c>
       <c r="F4" s="4">
         <f ca="1">TODAY()</f>
-        <v>46042</v>
+        <v>46051</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
@@ -19503,6 +19503,9 @@
       <c r="B34" t="s">
         <v>2181</v>
       </c>
+      <c r="V34" t="s">
+        <v>2181</v>
+      </c>
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A35" s="52" t="s">
@@ -19578,12 +19581,18 @@
       <c r="B38" t="s">
         <v>2226</v>
       </c>
+      <c r="V38" t="s">
+        <v>2226</v>
+      </c>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="52" t="s">
         <v>2392</v>
       </c>
       <c r="B39" t="s">
+        <v>2393</v>
+      </c>
+      <c r="V39" t="s">
         <v>2393</v>
       </c>
     </row>
@@ -20184,7 +20193,7 @@
         <v>1049</v>
       </c>
       <c r="B2" t="s">
-        <v>678</v>
+        <v>490</v>
       </c>
       <c r="C2" s="45">
         <v>5500100</v>
@@ -27385,7 +27394,7 @@
         <v>1968</v>
       </c>
       <c r="E2" t="s">
-        <v>246</v>
+        <v>490</v>
       </c>
       <c r="I2" t="s">
         <v>556</v>
@@ -27654,7 +27663,7 @@
         <v>1471</v>
       </c>
       <c r="E3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="F3" s="4">
         <v>45495</v>
@@ -31398,7 +31407,7 @@
         <v>0</v>
       </c>
       <c r="P32" t="s">
-        <v>658</v>
+        <v>2377</v>
       </c>
       <c r="AA32" t="s">
         <v>297</v>

</xml_diff>

<commit_message>
Adding missing screenshot update
</commit_message>
<xml_diff>
--- a/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
+++ b/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\testing\PIMS.Tests.Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46193B00-550F-4502-9BF0-5894803D468A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CA4A9A7-0774-46A3-9559-9FE00112EFED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="950" firstSheet="31" activeTab="31" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4420" uniqueCount="2447">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4422" uniqueCount="2449">
   <si>
     <t>FirstName</t>
   </si>
@@ -7424,6 +7424,12 @@
   </si>
   <si>
     <t>LMS220</t>
+  </si>
+  <si>
+    <t>Highway and Other Property Tabs</t>
+  </si>
+  <si>
+    <t>LMP16339</t>
   </si>
 </sst>
 </file>
@@ -10787,7 +10793,7 @@
       </c>
       <c r="N3" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="O3" s="4">
         <v>45318</v>
@@ -11031,7 +11037,7 @@
       </c>
       <c r="N5" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="O5" s="4">
         <v>45318</v>
@@ -11256,7 +11262,7 @@
       </c>
       <c r="N7" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="O7" s="4">
         <v>45318</v>
@@ -11829,7 +11835,7 @@
       </c>
       <c r="N12" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="O12" s="4">
         <v>45318</v>
@@ -12172,7 +12178,7 @@
       </c>
       <c r="N15" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="O15" s="4">
         <v>45318</v>
@@ -16957,7 +16963,7 @@
       </c>
       <c r="F4" s="4">
         <f ca="1">TODAY()</f>
-        <v>46070</v>
+        <v>46072</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
@@ -19005,7 +19011,7 @@
 
 <file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5E382B1-281B-4434-81AA-04C8D5F3D2FB}">
-  <dimension ref="A1:V40"/>
+  <dimension ref="A1:V41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="37.33203125" customWidth="1"/>
@@ -19644,6 +19650,14 @@
       </c>
       <c r="E40" t="s">
         <v>2446</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="A41" s="52" t="s">
+        <v>2447</v>
+      </c>
+      <c r="E41" t="s">
+        <v>2448</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improving waits on Test set
</commit_message>
<xml_diff>
--- a/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
+++ b/testing/PIMS.Tests.Automation/Data/PIMS_Testing_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SueT\projects\PSP\testing\PIMS.Tests.Automation\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD03F98A-7138-4FB8-86B6-E417405C8E00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4768597-B1D0-4672-A7BE-9076FCEC39CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="945" firstSheet="26" activeTab="26" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="945" firstSheet="30" activeTab="41" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AcquisitionChecklist" sheetId="22" r:id="rId1"/>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4511" uniqueCount="2490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4517" uniqueCount="2491">
   <si>
     <t>FirstName</t>
   </si>
@@ -7006,9 +7006,6 @@
     <t>675 davie</t>
   </si>
   <si>
-    <t>1253 bradshaw</t>
-  </si>
-  <si>
     <t>MF Property Digital Documents and Props Documents</t>
   </si>
   <si>
@@ -7168,9 +7165,6 @@
     <t>DisplayingList</t>
   </si>
   <si>
-    <t>015-279-511;028-175-913;018-353-690</t>
-  </si>
-  <si>
     <t>010-764-135;015-069-940;007-095-333</t>
   </si>
   <si>
@@ -7553,6 +7547,15 @@
   </si>
   <si>
     <t>013-215-469</t>
+  </si>
+  <si>
+    <t>Crossing Agreement</t>
+  </si>
+  <si>
+    <t>1818 West Mall</t>
+  </si>
+  <si>
+    <t>015-279-511;015-891-909;018-353-690</t>
   </si>
 </sst>
 </file>
@@ -8486,8 +8489,8 @@
     <col min="6" max="9" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="16" width="30.44140625" bestFit="1" customWidth="1"/>
     <col min="17" max="23" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="26" max="28" width="31.21875" customWidth="1"/>
+    <col min="24" max="25" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="26" max="28" width="31.33203125" customWidth="1"/>
     <col min="29" max="29" width="25.44140625" bestFit="1" customWidth="1"/>
     <col min="30" max="31" width="21.33203125" bestFit="1" customWidth="1"/>
     <col min="32" max="33" width="25.44140625" bestFit="1" customWidth="1"/>
@@ -8574,13 +8577,13 @@
         <v>2088</v>
       </c>
       <c r="Z1" s="19" t="s">
+        <v>2472</v>
+      </c>
+      <c r="AA1" s="19" t="s">
+        <v>2473</v>
+      </c>
+      <c r="AB1" s="19" t="s">
         <v>2474</v>
-      </c>
-      <c r="AA1" s="19" t="s">
-        <v>2475</v>
-      </c>
-      <c r="AB1" s="19" t="s">
-        <v>2476</v>
       </c>
       <c r="AC1" s="19" t="s">
         <v>2089</v>
@@ -9037,10 +9040,10 @@
         <v>1415</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>2442</v>
+        <v>2440</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>2443</v>
+        <v>2441</v>
       </c>
       <c r="X1" s="3" t="s">
         <v>1323</v>
@@ -9349,7 +9352,7 @@
       </c>
       <c r="F4" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" t="s">
@@ -10369,13 +10372,13 @@
     </row>
     <row r="17" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>2440</v>
+        <v>2438</v>
       </c>
       <c r="B17" t="s">
         <v>246</v>
       </c>
       <c r="H17" t="s">
-        <v>2441</v>
+        <v>2439</v>
       </c>
       <c r="J17" t="s">
         <v>1277</v>
@@ -10419,18 +10422,18 @@
     </row>
     <row r="18" spans="1:42" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>2449</v>
+        <v>2447</v>
       </c>
       <c r="B18" t="s">
         <v>246</v>
       </c>
       <c r="F18" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="G18" s="4"/>
       <c r="H18" t="s">
-        <v>2450</v>
+        <v>2448</v>
       </c>
       <c r="I18" t="s">
         <v>1331</v>
@@ -10791,7 +10794,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>2309</v>
+        <v>2308</v>
       </c>
       <c r="B17">
         <v>71</v>
@@ -10802,7 +10805,7 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>2352</v>
+        <v>2351</v>
       </c>
       <c r="B18">
         <v>71</v>
@@ -10813,12 +10816,12 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>2353</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>2354</v>
+        <v>2353</v>
       </c>
     </row>
   </sheetData>
@@ -10878,7 +10881,7 @@
         <v>501</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2392</v>
+        <v>2390</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>1867</v>
@@ -11195,7 +11198,7 @@
         <v>489</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>2393</v>
+        <v>2391</v>
       </c>
       <c r="I11" s="36"/>
       <c r="J11" s="36"/>
@@ -11410,7 +11413,7 @@
         <v>491</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>2394</v>
+        <v>2392</v>
       </c>
       <c r="I21" s="36"/>
       <c r="J21" s="36"/>
@@ -11648,7 +11651,7 @@
         <v>490</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>2395</v>
+        <v>2393</v>
       </c>
       <c r="I34" s="36"/>
       <c r="J34" s="36"/>
@@ -11878,7 +11881,7 @@
         <v>486</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>2396</v>
+        <v>2394</v>
       </c>
       <c r="I44" s="36"/>
       <c r="J44" s="36"/>
@@ -12048,7 +12051,7 @@
         <v>489</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>2397</v>
+        <v>2395</v>
       </c>
       <c r="I54" s="36"/>
       <c r="J54" s="36">
@@ -12241,7 +12244,7 @@
         <v>486</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>2398</v>
+        <v>2396</v>
       </c>
       <c r="I65" s="36"/>
       <c r="J65" s="36"/>
@@ -12363,7 +12366,7 @@
         <v>492</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>2399</v>
+        <v>2397</v>
       </c>
       <c r="I71" s="36"/>
       <c r="J71" s="36"/>
@@ -12389,7 +12392,7 @@
     </row>
     <row r="72" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>2310</v>
+        <v>2309</v>
       </c>
       <c r="B72" t="s">
         <v>710</v>
@@ -12398,12 +12401,12 @@
         <v>486</v>
       </c>
       <c r="AW72" t="s">
-        <v>2313</v>
+        <v>2312</v>
       </c>
     </row>
     <row r="73" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>2311</v>
+        <v>2310</v>
       </c>
       <c r="B73" t="s">
         <v>452</v>
@@ -12412,13 +12415,13 @@
         <v>487</v>
       </c>
       <c r="G73" t="s">
-        <v>2314</v>
+        <v>2313</v>
       </c>
       <c r="V73" t="s">
         <v>2211</v>
       </c>
       <c r="AU73" t="s">
-        <v>2315</v>
+        <v>2314</v>
       </c>
       <c r="BB73">
         <v>2025</v>
@@ -12426,7 +12429,7 @@
     </row>
     <row r="74" spans="1:54" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>2312</v>
+        <v>2311</v>
       </c>
       <c r="B74" t="s">
         <v>454</v>
@@ -12435,10 +12438,10 @@
         <v>488</v>
       </c>
       <c r="F74" t="s">
+        <v>2315</v>
+      </c>
+      <c r="U74" t="s">
         <v>2316</v>
-      </c>
-      <c r="U74" t="s">
-        <v>2317</v>
       </c>
     </row>
   </sheetData>
@@ -13563,10 +13566,10 @@
         <v>509</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>2415</v>
+        <v>2413</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>2416</v>
+        <v>2414</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>1626</v>
@@ -13671,7 +13674,7 @@
         <v>1619</v>
       </c>
       <c r="AV1" s="3" t="s">
-        <v>2459</v>
+        <v>2457</v>
       </c>
       <c r="AW1" s="3" t="s">
         <v>1735</v>
@@ -14068,7 +14071,7 @@
         <v>45495</v>
       </c>
       <c r="I3" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J3" s="4">
         <v>44614</v>
@@ -14080,7 +14083,7 @@
         <v>1946</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>2417</v>
+        <v>2415</v>
       </c>
       <c r="N3" s="8">
         <v>4</v>
@@ -14088,8 +14091,14 @@
       <c r="O3" s="8">
         <v>1</v>
       </c>
+      <c r="Q3" t="s">
+        <v>192</v>
+      </c>
       <c r="R3" t="s">
         <v>634</v>
+      </c>
+      <c r="T3" t="s">
+        <v>2488</v>
       </c>
       <c r="V3" t="s">
         <v>1725</v>
@@ -14438,13 +14447,13 @@
     </row>
     <row r="6" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>2376</v>
+        <v>2374</v>
       </c>
       <c r="E6" t="s">
         <v>487</v>
       </c>
       <c r="I6" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J6" s="4">
         <v>45064</v>
@@ -14464,7 +14473,7 @@
         <v>190</v>
       </c>
       <c r="R6" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T6" t="s">
         <v>1682</v>
@@ -14823,7 +14832,7 @@
         <v>487</v>
       </c>
       <c r="I9" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J9" s="4">
         <v>45209</v>
@@ -14948,7 +14957,7 @@
         <v>487</v>
       </c>
       <c r="I10" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J10" s="4">
         <v>45209</v>
@@ -15079,7 +15088,7 @@
         <v>190</v>
       </c>
       <c r="R11" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T11" t="s">
         <v>1682</v>
@@ -15201,7 +15210,7 @@
         <v>190</v>
       </c>
       <c r="R12" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T12" t="s">
         <v>1682</v>
@@ -15326,7 +15335,7 @@
         <v>190</v>
       </c>
       <c r="R13" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T13" t="s">
         <v>1682</v>
@@ -15448,7 +15457,7 @@
         <v>190</v>
       </c>
       <c r="R14" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T14" t="s">
         <v>1682</v>
@@ -15570,7 +15579,7 @@
         <v>190</v>
       </c>
       <c r="R15" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T15" t="s">
         <v>1682</v>
@@ -15698,7 +15707,7 @@
         <v>190</v>
       </c>
       <c r="R16" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T16" t="s">
         <v>1682</v>
@@ -15825,7 +15834,7 @@
         <v>190</v>
       </c>
       <c r="R17" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T17" t="s">
         <v>1682</v>
@@ -15952,7 +15961,7 @@
         <v>190</v>
       </c>
       <c r="R18" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T18" t="s">
         <v>1682</v>
@@ -16053,7 +16062,7 @@
     </row>
     <row r="19" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>2350</v>
+        <v>2349</v>
       </c>
       <c r="B19" t="s">
         <v>980</v>
@@ -16068,7 +16077,7 @@
         <v>487</v>
       </c>
       <c r="I19" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J19" s="4">
         <v>45209</v>
@@ -16187,13 +16196,13 @@
     </row>
     <row r="20" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>2351</v>
+        <v>2350</v>
       </c>
       <c r="E20" t="s">
         <v>487</v>
       </c>
       <c r="I20" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="N20" s="8">
         <v>0</v>
@@ -16306,7 +16315,7 @@
     </row>
     <row r="21" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>2364</v>
+        <v>2362</v>
       </c>
       <c r="E21" t="s">
         <v>246</v>
@@ -16441,7 +16450,7 @@
     </row>
     <row r="22" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>2369</v>
+        <v>2367</v>
       </c>
       <c r="E22" t="s">
         <v>246</v>
@@ -16554,7 +16563,7 @@
     </row>
     <row r="23" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>2365</v>
+        <v>2363</v>
       </c>
       <c r="E23" t="s">
         <v>246</v>
@@ -16689,7 +16698,7 @@
     </row>
     <row r="24" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>2366</v>
+        <v>2364</v>
       </c>
       <c r="E24" t="s">
         <v>246</v>
@@ -16824,7 +16833,7 @@
     </row>
     <row r="25" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>2370</v>
+        <v>2368</v>
       </c>
       <c r="E25" t="s">
         <v>246</v>
@@ -16942,7 +16951,7 @@
     </row>
     <row r="26" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>2367</v>
+        <v>2365</v>
       </c>
       <c r="E26" t="s">
         <v>246</v>
@@ -17157,7 +17166,7 @@
     </row>
     <row r="27" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>2371</v>
+        <v>2369</v>
       </c>
       <c r="E27" t="s">
         <v>246</v>
@@ -17283,7 +17292,7 @@
     </row>
     <row r="28" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>2368</v>
+        <v>2366</v>
       </c>
       <c r="E28" t="s">
         <v>246</v>
@@ -17421,7 +17430,7 @@
     </row>
     <row r="29" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>2372</v>
+        <v>2370</v>
       </c>
       <c r="F29" s="4"/>
       <c r="J29" s="4"/>
@@ -17536,7 +17545,7 @@
     </row>
     <row r="30" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>2373</v>
+        <v>2371</v>
       </c>
       <c r="E30" t="s">
         <v>246</v>
@@ -17671,7 +17680,7 @@
     </row>
     <row r="31" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>2374</v>
+        <v>2372</v>
       </c>
       <c r="F31" s="4"/>
       <c r="J31" s="4"/>
@@ -17783,7 +17792,7 @@
     </row>
     <row r="32" spans="1:90" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>2375</v>
+        <v>2373</v>
       </c>
       <c r="N32" s="8">
         <v>0</v>
@@ -17792,7 +17801,7 @@
         <v>0</v>
       </c>
       <c r="R32" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="AC32" t="s">
         <v>295</v>
@@ -17893,7 +17902,7 @@
         <v>487</v>
       </c>
       <c r="I33" t="s">
-        <v>2320</v>
+        <v>2319</v>
       </c>
       <c r="J33" s="4">
         <v>45064</v>
@@ -17913,7 +17922,7 @@
         <v>190</v>
       </c>
       <c r="R33" t="s">
-        <v>2340</v>
+        <v>2339</v>
       </c>
       <c r="T33" t="s">
         <v>1682</v>
@@ -18006,13 +18015,13 @@
     </row>
     <row r="34" spans="1:89" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>2377</v>
+        <v>2375</v>
       </c>
       <c r="E34" t="s">
         <v>487</v>
       </c>
       <c r="I34" t="s">
-        <v>2320</v>
+        <v>567</v>
       </c>
       <c r="J34" s="4">
         <v>45064</v>
@@ -20352,7 +20361,7 @@
         <v>2165</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>2407</v>
+        <v>2405</v>
       </c>
       <c r="J1" s="3" t="s">
         <v>2166</v>
@@ -20361,7 +20370,7 @@
         <v>2167</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>2408</v>
+        <v>2406</v>
       </c>
       <c r="M1" s="3" t="s">
         <v>2168</v>
@@ -20370,16 +20379,16 @@
         <v>2169</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>2409</v>
+        <v>2407</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>2410</v>
+        <v>2408</v>
       </c>
       <c r="Q1" s="3" t="s">
         <v>2170</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>2359</v>
+        <v>2358</v>
       </c>
       <c r="S1" s="3" t="s">
         <v>2274</v>
@@ -20429,10 +20438,10 @@
         <v>2</v>
       </c>
       <c r="O2" t="s">
+        <v>2409</v>
+      </c>
+      <c r="P2" t="s">
         <v>2411</v>
-      </c>
-      <c r="P2" t="s">
-        <v>2413</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -20488,10 +20497,10 @@
         <v>1</v>
       </c>
       <c r="O3" t="s">
+        <v>2410</v>
+      </c>
+      <c r="P3" t="s">
         <v>2412</v>
-      </c>
-      <c r="P3" t="s">
-        <v>2414</v>
       </c>
       <c r="Q3">
         <v>0</v>
@@ -20764,13 +20773,13 @@
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>2357</v>
+        <v>2356</v>
       </c>
       <c r="B12" t="s">
         <v>487</v>
       </c>
       <c r="G12" t="s">
-        <v>2358</v>
+        <v>2357</v>
       </c>
       <c r="J12" t="s">
         <v>1754</v>
@@ -21198,15 +21207,15 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>2349</v>
+        <v>2348</v>
       </c>
       <c r="B14" t="s">
-        <v>2347</v>
+        <v>2346</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>2348</v>
+        <v>2347</v>
       </c>
       <c r="B15" t="s">
         <v>2226</v>
@@ -22858,7 +22867,7 @@
     <col min="23" max="23" width="32.33203125" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="22.109375" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="20.6640625" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="17.44140625" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="19.44140625" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -22953,13 +22962,13 @@
         <v>1549</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>2401</v>
+        <v>2399</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>2455</v>
+        <v>2453</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>2456</v>
+        <v>2454</v>
       </c>
       <c r="AA1" s="3" t="s">
         <v>1550</v>
@@ -22974,19 +22983,19 @@
         <v>1553</v>
       </c>
       <c r="AE1" s="3" t="s">
+        <v>2416</v>
+      </c>
+      <c r="AF1" s="3" t="s">
+        <v>2417</v>
+      </c>
+      <c r="AG1" s="3" t="s">
         <v>2418</v>
       </c>
-      <c r="AF1" s="3" t="s">
+      <c r="AH1" s="3" t="s">
         <v>2419</v>
       </c>
-      <c r="AG1" s="3" t="s">
+      <c r="AI1" s="3" t="s">
         <v>2420</v>
-      </c>
-      <c r="AH1" s="3" t="s">
-        <v>2421</v>
-      </c>
-      <c r="AI1" s="3" t="s">
-        <v>2422</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.3">
@@ -23002,6 +23011,9 @@
       <c r="M2">
         <v>0</v>
       </c>
+      <c r="O2" t="s">
+        <v>190</v>
+      </c>
       <c r="AB2" s="16" t="b">
         <v>1</v>
       </c>
@@ -23142,7 +23154,7 @@
         <v>1243</v>
       </c>
       <c r="W4" t="s">
-        <v>2344</v>
+        <v>2343</v>
       </c>
       <c r="AA4" s="30">
         <v>65.898600000000002</v>
@@ -23201,13 +23213,13 @@
         <v>694</v>
       </c>
       <c r="X5" t="s">
-        <v>2452</v>
+        <v>2450</v>
       </c>
       <c r="Y5" t="s">
-        <v>2457</v>
+        <v>2455</v>
       </c>
       <c r="Z5" t="s">
-        <v>2458</v>
+        <v>2456</v>
       </c>
       <c r="AA5" s="30">
         <v>89.87</v>
@@ -23222,13 +23234,13 @@
         <v>670</v>
       </c>
       <c r="AE5" t="s">
-        <v>2453</v>
+        <v>2451</v>
       </c>
       <c r="AF5" t="s">
-        <v>2404</v>
+        <v>2402</v>
       </c>
       <c r="AG5" t="s">
-        <v>2454</v>
+        <v>2452</v>
       </c>
       <c r="AH5">
         <v>0</v>
@@ -23310,7 +23322,7 @@
     </row>
     <row r="7" spans="1:35" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>2425</v>
+        <v>2423</v>
       </c>
       <c r="B7" t="s">
         <v>1568</v>
@@ -23321,11 +23333,20 @@
       <c r="M7">
         <v>0</v>
       </c>
+      <c r="O7" t="s">
+        <v>190</v>
+      </c>
+      <c r="P7" t="s">
+        <v>1555</v>
+      </c>
+      <c r="AA7" s="30">
+        <v>65.898600000000002</v>
+      </c>
       <c r="AB7" s="16" t="b">
-        <v>0</v>
-      </c>
-      <c r="AC7">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="AC7" s="32" t="s">
+        <v>1597</v>
       </c>
       <c r="AD7" t="s">
         <v>268</v>
@@ -23417,8 +23438,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="30.6640625" bestFit="1" customWidth="1"/>
@@ -23429,67 +23449,67 @@
         <v>104</v>
       </c>
       <c r="B1" s="3" t="s">
+        <v>2475</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2422</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>2476</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>2477</v>
       </c>
-      <c r="C1" s="3" t="s">
-        <v>2424</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>2478</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>2479</v>
-      </c>
       <c r="F1" s="3" t="s">
-        <v>2423</v>
+        <v>2421</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>2424</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2478</v>
+      </c>
+      <c r="C2" t="s">
         <v>2426</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2480</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2428</v>
       </c>
       <c r="D2" t="s">
         <v>246</v>
       </c>
       <c r="E2" t="s">
-        <v>2404</v>
+        <v>2402</v>
       </c>
       <c r="F2" t="s">
-        <v>2430</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>2426</v>
+        <v>2424</v>
       </c>
       <c r="B3" t="s">
-        <v>2481</v>
+        <v>2479</v>
       </c>
       <c r="C3" t="s">
-        <v>2429</v>
+        <v>2427</v>
       </c>
       <c r="D3" t="s">
         <v>246</v>
       </c>
       <c r="E3" t="s">
-        <v>2484</v>
+        <v>2482</v>
       </c>
       <c r="F3" t="s">
-        <v>2431</v>
+        <v>2429</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>2426</v>
+        <v>2424</v>
       </c>
       <c r="B4" t="s">
-        <v>2482</v>
+        <v>2480</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -23498,30 +23518,30 @@
         <v>247</v>
       </c>
       <c r="E4" t="s">
-        <v>2485</v>
+        <v>2483</v>
       </c>
       <c r="F4" t="s">
-        <v>2432</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>2425</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2481</v>
+      </c>
+      <c r="C5" t="s">
         <v>2427</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2483</v>
-      </c>
-      <c r="C5" t="s">
-        <v>2429</v>
       </c>
       <c r="D5" t="s">
         <v>247</v>
       </c>
       <c r="E5" t="s">
-        <v>2486</v>
+        <v>2484</v>
       </c>
       <c r="F5" t="s">
-        <v>2433</v>
+        <v>2431</v>
       </c>
     </row>
   </sheetData>
@@ -23874,7 +23894,7 @@
         <v>1161</v>
       </c>
       <c r="D2" t="s">
-        <v>2383</v>
+        <v>2381</v>
       </c>
       <c r="E2" t="s">
         <v>1185</v>
@@ -23889,7 +23909,7 @@
         <v>2125</v>
       </c>
       <c r="J2" t="s">
-        <v>2378</v>
+        <v>2376</v>
       </c>
       <c r="K2" t="s">
         <v>1167</v>
@@ -23927,7 +23947,7 @@
         <v>1162</v>
       </c>
       <c r="D3" t="s">
-        <v>2384</v>
+        <v>2382</v>
       </c>
       <c r="E3" t="s">
         <v>1163</v>
@@ -23942,7 +23962,7 @@
         <v>1166</v>
       </c>
       <c r="J3" t="s">
-        <v>2379</v>
+        <v>2377</v>
       </c>
       <c r="K3" t="s">
         <v>2124</v>
@@ -23995,7 +24015,7 @@
         <v>1195</v>
       </c>
       <c r="J4" t="s">
-        <v>2487</v>
+        <v>2485</v>
       </c>
       <c r="K4" t="s">
         <v>1197</v>
@@ -24033,7 +24053,7 @@
         <v>1250</v>
       </c>
       <c r="D5" t="s">
-        <v>2385</v>
+        <v>2383</v>
       </c>
       <c r="E5" t="s">
         <v>1185</v>
@@ -24048,7 +24068,7 @@
         <v>2191</v>
       </c>
       <c r="J5" t="s">
-        <v>2380</v>
+        <v>2378</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -24095,13 +24115,13 @@
         <v>2301</v>
       </c>
       <c r="J6" t="s">
-        <v>2381</v>
+        <v>2379</v>
       </c>
       <c r="K6" t="s">
         <v>2302</v>
       </c>
       <c r="L6" t="s">
-        <v>2460</v>
+        <v>2458</v>
       </c>
       <c r="M6">
         <v>3</v>
@@ -24151,10 +24171,10 @@
         <v>2272</v>
       </c>
       <c r="J7" t="s">
-        <v>2382</v>
+        <v>2380</v>
       </c>
       <c r="K7" t="s">
-        <v>2386</v>
+        <v>2384</v>
       </c>
       <c r="L7" s="14" t="s">
         <v>2280</v>
@@ -24201,13 +24221,13 @@
         <v>2271</v>
       </c>
       <c r="I8" t="s">
+        <v>2385</v>
+      </c>
+      <c r="J8" t="s">
+        <v>2386</v>
+      </c>
+      <c r="K8" t="s">
         <v>2387</v>
-      </c>
-      <c r="J8" t="s">
-        <v>2388</v>
-      </c>
-      <c r="K8" t="s">
-        <v>2389</v>
       </c>
       <c r="L8" t="s">
         <v>2281</v>
@@ -24630,10 +24650,10 @@
         <v>770</v>
       </c>
       <c r="AH1" s="38" t="s">
-        <v>2402</v>
+        <v>2400</v>
       </c>
       <c r="AI1" s="38" t="s">
-        <v>2403</v>
+        <v>2401</v>
       </c>
       <c r="AJ1" s="38" t="s">
         <v>1303</v>
@@ -24782,10 +24802,10 @@
         <v>768</v>
       </c>
       <c r="AH2" t="s">
-        <v>2404</v>
+        <v>2402</v>
       </c>
       <c r="AI2" t="s">
-        <v>2405</v>
+        <v>2403</v>
       </c>
       <c r="AJ2">
         <v>15</v>
@@ -24875,7 +24895,7 @@
       </c>
       <c r="N3" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="O3" s="4">
         <v>45318</v>
@@ -24923,10 +24943,10 @@
         <v>981</v>
       </c>
       <c r="AH3" t="s">
-        <v>2451</v>
+        <v>2449</v>
       </c>
       <c r="AI3" t="s">
-        <v>2406</v>
+        <v>2404</v>
       </c>
       <c r="AJ3">
         <v>0</v>
@@ -25119,7 +25139,7 @@
       </c>
       <c r="N5" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="O5" s="4">
         <v>45318</v>
@@ -25344,7 +25364,7 @@
       </c>
       <c r="N7" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="O7" s="4">
         <v>45318</v>
@@ -25917,7 +25937,7 @@
       </c>
       <c r="N12" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="O12" s="4">
         <v>45318</v>
@@ -26260,7 +26280,7 @@
       </c>
       <c r="N15" s="4">
         <f ca="1">TODAY()</f>
-        <v>46100</v>
+        <v>46125</v>
       </c>
       <c r="O15" s="4">
         <v>45318</v>
@@ -27888,13 +27908,13 @@
         <v>239</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>2321</v>
+        <v>2320</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>1471</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>2322</v>
+        <v>2321</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>2250</v>
@@ -27921,22 +27941,22 @@
         <v>2257</v>
       </c>
       <c r="Q1" s="3" t="s">
+        <v>2322</v>
+      </c>
+      <c r="R1" s="3" t="s">
         <v>2323</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>2324</v>
       </c>
-      <c r="S1" s="3" t="s">
+      <c r="T1" s="3" t="s">
         <v>2325</v>
       </c>
-      <c r="T1" s="3" t="s">
-        <v>2326</v>
-      </c>
       <c r="U1" s="3" t="s">
-        <v>2400</v>
+        <v>2398</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>2360</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
@@ -27947,7 +27967,7 @@
         <v>4361431</v>
       </c>
       <c r="D2" t="s">
-        <v>2307</v>
+        <v>2489</v>
       </c>
       <c r="I2">
         <v>48</v>
@@ -27974,7 +27994,7 @@
         <v>2259</v>
       </c>
       <c r="V2" s="14" t="s">
-        <v>2361</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.3">
@@ -27982,7 +28002,7 @@
         <v>325</v>
       </c>
       <c r="H3" t="s">
-        <v>2342</v>
+        <v>2341</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
@@ -27990,7 +28010,7 @@
         <v>278</v>
       </c>
       <c r="D4" t="s">
-        <v>2341</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
@@ -27998,7 +28018,7 @@
         <v>276</v>
       </c>
       <c r="B5" t="s">
-        <v>2343</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.3">
@@ -28090,7 +28110,7 @@
         <v>1289</v>
       </c>
       <c r="G12" t="s">
-        <v>2338</v>
+        <v>2337</v>
       </c>
       <c r="I12">
         <v>49</v>
@@ -28117,10 +28137,10 @@
         <v>2259</v>
       </c>
       <c r="Q12" t="s">
-        <v>2339</v>
+        <v>2338</v>
       </c>
       <c r="V12" t="s">
-        <v>2363</v>
+        <v>2361</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.3">
@@ -28158,19 +28178,19 @@
         <v>1821391</v>
       </c>
       <c r="D16" t="s">
-        <v>2329</v>
+        <v>2328</v>
       </c>
       <c r="E16" t="s">
         <v>1714</v>
       </c>
       <c r="H16" t="s">
-        <v>2328</v>
+        <v>2327</v>
       </c>
       <c r="Q16" t="s">
-        <v>2327</v>
+        <v>2326</v>
       </c>
       <c r="V16" t="s">
-        <v>2362</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.3">
@@ -28268,13 +28288,13 @@
         <v>1727</v>
       </c>
       <c r="F26" t="s">
+        <v>2334</v>
+      </c>
+      <c r="H26" t="s">
         <v>2335</v>
       </c>
-      <c r="H26" t="s">
-        <v>2336</v>
-      </c>
       <c r="V26" t="s">
-        <v>2461</v>
+        <v>2459</v>
       </c>
     </row>
     <row r="27" spans="1:22" x14ac:dyDescent="0.3">
@@ -28311,7 +28331,7 @@
         <v>1308</v>
       </c>
       <c r="H28" t="s">
-        <v>2317</v>
+        <v>2316</v>
       </c>
     </row>
     <row r="29" spans="1:22" x14ac:dyDescent="0.3">
@@ -28319,7 +28339,7 @@
         <v>1309</v>
       </c>
       <c r="F29" t="s">
-        <v>2337</v>
+        <v>2336</v>
       </c>
     </row>
     <row r="30" spans="1:22" x14ac:dyDescent="0.3">
@@ -28353,10 +28373,10 @@
         <v>2137</v>
       </c>
       <c r="B32" t="s">
-        <v>2489</v>
+        <v>2487</v>
       </c>
       <c r="V32" t="s">
-        <v>2489</v>
+        <v>2487</v>
       </c>
     </row>
     <row r="33" spans="1:22" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -28367,7 +28387,7 @@
         <v>2141</v>
       </c>
       <c r="F33" t="s">
-        <v>2334</v>
+        <v>2333</v>
       </c>
       <c r="V33" s="14" t="s">
         <v>2141</v>
@@ -28395,7 +28415,7 @@
         <v>90172682</v>
       </c>
       <c r="D35" t="s">
-        <v>2390</v>
+        <v>2388</v>
       </c>
       <c r="E35" t="s">
         <v>2194</v>
@@ -28425,7 +28445,7 @@
         <v>2259</v>
       </c>
       <c r="V35" t="s">
-        <v>2391</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.3">
@@ -28444,15 +28464,15 @@
         <v>2305</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>2488</v>
+        <v>2486</v>
       </c>
       <c r="V37" s="14" t="s">
-        <v>2488</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="38" spans="1:22" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A38" s="52" t="s">
-        <v>2308</v>
+        <v>2307</v>
       </c>
       <c r="B38" t="s">
         <v>2193</v>
@@ -28463,37 +28483,37 @@
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A39" s="52" t="s">
+        <v>2354</v>
+      </c>
+      <c r="B39" t="s">
         <v>2355</v>
       </c>
-      <c r="B39" t="s">
-        <v>2356</v>
-      </c>
       <c r="V39" t="s">
-        <v>2356</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A40" s="52" t="s">
-        <v>2434</v>
+        <v>2432</v>
       </c>
       <c r="E40" t="s">
-        <v>2435</v>
+        <v>2433</v>
       </c>
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A41" s="52" t="s">
-        <v>2436</v>
+        <v>2434</v>
       </c>
       <c r="E41" t="s">
-        <v>2437</v>
+        <v>2435</v>
       </c>
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A42" s="52" t="s">
-        <v>2438</v>
+        <v>2436</v>
       </c>
       <c r="B42" t="s">
-        <v>2439</v>
+        <v>2437</v>
       </c>
     </row>
   </sheetData>
@@ -30656,7 +30676,7 @@
         <v>650</v>
       </c>
       <c r="B2" t="s">
-        <v>2318</v>
+        <v>2317</v>
       </c>
       <c r="C2" t="s">
         <v>250</v>
@@ -30746,7 +30766,7 @@
         <v>863</v>
       </c>
       <c r="B8" t="s">
-        <v>2318</v>
+        <v>2317</v>
       </c>
       <c r="C8" t="s">
         <v>864</v>
@@ -30777,7 +30797,7 @@
         <v>1060</v>
       </c>
       <c r="B10" t="s">
-        <v>2318</v>
+        <v>2317</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>1061</v>
@@ -30791,7 +30811,7 @@
         <v>1209</v>
       </c>
       <c r="B11" t="s">
-        <v>2318</v>
+        <v>2317</v>
       </c>
       <c r="C11" t="s">
         <v>2102</v>
@@ -30819,7 +30839,7 @@
         <v>1312</v>
       </c>
       <c r="B13" t="s">
-        <v>2318</v>
+        <v>2317</v>
       </c>
       <c r="C13" t="s">
         <v>1313</v>
@@ -30833,7 +30853,7 @@
         <v>1312</v>
       </c>
       <c r="B14" t="s">
-        <v>2319</v>
+        <v>2318</v>
       </c>
       <c r="C14" t="s">
         <v>1314</v>
@@ -31776,8 +31796,8 @@
     <col min="4" max="4" width="46.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="52.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.21875" customWidth="1"/>
+    <col min="7" max="7" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.33203125" customWidth="1"/>
     <col min="9" max="9" width="50.6640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.6640625" bestFit="1" customWidth="1"/>
@@ -31855,10 +31875,10 @@
         <v>487</v>
       </c>
       <c r="H2" t="s">
-        <v>2463</v>
+        <v>2461</v>
       </c>
       <c r="I2" t="s">
-        <v>2471</v>
+        <v>2469</v>
       </c>
       <c r="J2" s="4">
         <v>44440</v>
@@ -31902,10 +31922,10 @@
         <v>487</v>
       </c>
       <c r="H3" t="s">
-        <v>2464</v>
+        <v>2462</v>
       </c>
       <c r="I3" t="s">
-        <v>2472</v>
+        <v>2470</v>
       </c>
       <c r="J3" s="4">
         <v>44806</v>
@@ -31946,10 +31966,10 @@
         <v>492</v>
       </c>
       <c r="G4" t="s">
-        <v>2462</v>
+        <v>2460</v>
       </c>
       <c r="H4" t="s">
-        <v>2465</v>
+        <v>2463</v>
       </c>
       <c r="I4" t="s">
         <v>796</v>
@@ -31993,7 +32013,7 @@
         <v>487</v>
       </c>
       <c r="H5" t="s">
-        <v>2466</v>
+        <v>2464</v>
       </c>
       <c r="I5" t="s">
         <v>797</v>
@@ -32037,7 +32057,7 @@
         <v>487</v>
       </c>
       <c r="H6" t="s">
-        <v>2467</v>
+        <v>2465</v>
       </c>
       <c r="I6" t="s">
         <v>794</v>
@@ -32081,7 +32101,7 @@
         <v>487</v>
       </c>
       <c r="H7" t="s">
-        <v>2467</v>
+        <v>2465</v>
       </c>
       <c r="I7" t="s">
         <v>794</v>
@@ -32125,10 +32145,10 @@
         <v>487</v>
       </c>
       <c r="H8" t="s">
-        <v>2468</v>
+        <v>2466</v>
       </c>
       <c r="I8" t="s">
-        <v>2473</v>
+        <v>2471</v>
       </c>
       <c r="J8" s="4">
         <v>45265</v>
@@ -32154,25 +32174,25 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>2444</v>
+        <v>2442</v>
       </c>
       <c r="B9" t="s">
         <v>487</v>
       </c>
       <c r="D9" t="s">
+        <v>2444</v>
+      </c>
+      <c r="E9" t="s">
         <v>2446</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2448</v>
       </c>
       <c r="F9" t="s">
         <v>487</v>
       </c>
       <c r="H9" t="s">
-        <v>2469</v>
+        <v>2467</v>
       </c>
       <c r="I9" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="J9" s="4">
         <v>45658</v>
@@ -32198,25 +32218,25 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>2445</v>
+        <v>2443</v>
       </c>
       <c r="B10" t="s">
         <v>487</v>
       </c>
       <c r="D10" t="s">
-        <v>2447</v>
+        <v>2445</v>
       </c>
       <c r="E10" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="F10" t="s">
         <v>487</v>
       </c>
       <c r="H10" t="s">
-        <v>2470</v>
+        <v>2468</v>
       </c>
       <c r="I10" t="s">
-        <v>2448</v>
+        <v>2446</v>
       </c>
       <c r="J10" s="4">
         <v>45690</v>
@@ -32390,7 +32410,7 @@
         <v>858</v>
       </c>
       <c r="P2" t="s">
-        <v>2330</v>
+        <v>2329</v>
       </c>
       <c r="Q2" t="s">
         <v>2104</v>
@@ -32431,7 +32451,7 @@
         <v>974</v>
       </c>
       <c r="P3" t="s">
-        <v>2331</v>
+        <v>2330</v>
       </c>
       <c r="Q3" t="s">
         <v>2105</v>
@@ -32493,7 +32513,7 @@
         <v>858</v>
       </c>
       <c r="P4" t="s">
-        <v>2332</v>
+        <v>2331</v>
       </c>
       <c r="Q4" t="s">
         <v>2102</v>
@@ -32655,7 +32675,7 @@
         <v>858</v>
       </c>
       <c r="P7" t="s">
-        <v>2333</v>
+        <v>2332</v>
       </c>
       <c r="Q7" t="s">
         <v>2106</v>
@@ -32789,7 +32809,7 @@
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>2345</v>
+        <v>2344</v>
       </c>
       <c r="B10" s="37"/>
       <c r="E10" t="s">
@@ -32802,7 +32822,7 @@
         <v>45569</v>
       </c>
       <c r="K10" t="s">
-        <v>2346</v>
+        <v>2345</v>
       </c>
       <c r="L10" t="s">
         <v>1530</v>

</xml_diff>